<commit_message>
mejoras en deteccion de cedula, reset de placeholders y estabilidad
</commit_message>
<xml_diff>
--- a/data/Bases de datos Prototipo Copiloto admisión.xlsx
+++ b/data/Bases de datos Prototipo Copiloto admisión.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2EDFEC27-0E2B-4C1D-9002-A4A7AAF287EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Juan Casanova\Documents\College\8thSemester\IA\proyects\medical-copilot\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93671A15-8000-4E05-94AA-7715E02D7EBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1920" yWindow="756" windowWidth="18900" windowHeight="12204" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Servicios" sheetId="1" r:id="rId1"/>
@@ -1468,7 +1473,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -1735,9 +1740,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1775,7 +1780,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1881,7 +1886,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2023,7 +2028,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2032,16 +2037,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I110"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
-    <col min="2" max="2" width="22.42578125" customWidth="1"/>
-    <col min="3" max="3" width="19.42578125" customWidth="1"/>
+    <col min="2" max="2" width="22.44140625" customWidth="1"/>
+    <col min="3" max="3" width="19.44140625" customWidth="1"/>
     <col min="4" max="4" width="55" customWidth="1"/>
-    <col min="5" max="5" width="38.7109375" customWidth="1"/>
-    <col min="6" max="6" width="35.28515625" customWidth="1"/>
-    <col min="7" max="7" width="24.85546875" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" customWidth="1"/>
+    <col min="5" max="5" width="38.6640625" customWidth="1"/>
+    <col min="6" max="6" width="35.33203125" customWidth="1"/>
+    <col min="7" max="7" width="24.88671875" customWidth="1"/>
+    <col min="9" max="9" width="13.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -4916,28 +4921,28 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0E0A4C3-E7CF-436B-A59A-4EBD0F1D8B18}">
   <dimension ref="A1:AD7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" style="12" customWidth="1"/>
-    <col min="2" max="4" width="9.140625" style="12"/>
-    <col min="5" max="5" width="16.5703125" style="12" customWidth="1"/>
-    <col min="6" max="6" width="20.28515625" style="12" customWidth="1"/>
-    <col min="7" max="9" width="9.140625" style="12"/>
-    <col min="10" max="10" width="10.85546875" style="12" bestFit="1" customWidth="1"/>
-    <col min="11" max="18" width="9.140625" style="12"/>
-    <col min="19" max="19" width="12.7109375" style="12" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.42578125" style="12" customWidth="1"/>
+    <col min="1" max="1" width="12.5546875" style="12" customWidth="1"/>
+    <col min="2" max="4" width="9.109375" style="12"/>
+    <col min="5" max="5" width="16.5546875" style="12" customWidth="1"/>
+    <col min="6" max="6" width="20.33203125" style="12" customWidth="1"/>
+    <col min="7" max="9" width="9.109375" style="12"/>
+    <col min="10" max="10" width="10.88671875" style="12" bestFit="1" customWidth="1"/>
+    <col min="11" max="18" width="9.109375" style="12"/>
+    <col min="19" max="19" width="12.6640625" style="12" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.44140625" style="12" customWidth="1"/>
     <col min="21" max="21" width="13" style="12" customWidth="1"/>
-    <col min="22" max="23" width="9.140625" style="12"/>
-    <col min="24" max="24" width="14.28515625" style="12" customWidth="1"/>
-    <col min="25" max="25" width="11.7109375" style="12" customWidth="1"/>
-    <col min="26" max="27" width="12.42578125" style="12" customWidth="1"/>
-    <col min="28" max="28" width="13.85546875" style="12" customWidth="1"/>
-    <col min="29" max="29" width="46.28515625" style="12" customWidth="1"/>
-    <col min="30" max="16384" width="9.140625" style="12"/>
+    <col min="22" max="23" width="9.109375" style="12"/>
+    <col min="24" max="24" width="14.33203125" style="12" customWidth="1"/>
+    <col min="25" max="25" width="11.6640625" style="12" customWidth="1"/>
+    <col min="26" max="27" width="12.44140625" style="12" customWidth="1"/>
+    <col min="28" max="28" width="13.88671875" style="12" customWidth="1"/>
+    <col min="29" max="29" width="46.33203125" style="12" customWidth="1"/>
+    <col min="30" max="16384" width="9.109375" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" s="11" customFormat="1" ht="53.25">
+    <row r="1" spans="1:30" s="11" customFormat="1" ht="69">
       <c r="A1" s="22" t="s">
         <v>54</v>
       </c>
@@ -5115,7 +5120,7 @@
       </c>
       <c r="AD2" s="21"/>
     </row>
-    <row r="3" spans="1:30" ht="27">
+    <row r="3" spans="1:30" ht="27.6">
       <c r="A3" s="24" t="s">
         <v>107</v>
       </c>
@@ -5128,7 +5133,7 @@
         <v>86</v>
       </c>
       <c r="F3" s="25">
-        <v>27998946</v>
+        <v>1127668334</v>
       </c>
       <c r="G3" s="24" t="s">
         <v>109</v>
@@ -5451,7 +5456,7 @@
       </c>
       <c r="AD6" s="21"/>
     </row>
-    <row r="7" spans="1:30" ht="27">
+    <row r="7" spans="1:30" ht="27.6">
       <c r="A7" s="24" t="s">
         <v>142</v>
       </c>
@@ -5553,11 +5558,11 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{333480C1-FAC5-4EC7-9474-8E7E196759BA}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="28.42578125" customWidth="1"/>
+    <col min="1" max="1" width="28.44140625" customWidth="1"/>
     <col min="2" max="2" width="33" customWidth="1"/>
-    <col min="3" max="3" width="56.28515625" customWidth="1"/>
+    <col min="3" max="3" width="56.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -5587,7 +5592,7 @@
         <v>86</v>
       </c>
       <c r="B3" s="30">
-        <v>27998946</v>
+        <v>1127668334</v>
       </c>
       <c r="C3" s="31" t="s">
         <v>106</v>
@@ -5645,14 +5650,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7275EB94-9A20-4D60-9ACC-F8C9BBA6218D}">
   <dimension ref="A1:H16"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="25.7109375" customWidth="1"/>
-    <col min="3" max="3" width="14.85546875" customWidth="1"/>
-    <col min="4" max="4" width="32.42578125" customWidth="1"/>
-    <col min="5" max="5" width="18.7109375" customWidth="1"/>
-    <col min="6" max="6" width="29.7109375" customWidth="1"/>
-    <col min="7" max="7" width="18.7109375" customWidth="1"/>
+    <col min="1" max="1" width="25.6640625" customWidth="1"/>
+    <col min="3" max="3" width="14.88671875" customWidth="1"/>
+    <col min="4" max="4" width="32.44140625" customWidth="1"/>
+    <col min="5" max="5" width="18.6640625" customWidth="1"/>
+    <col min="6" max="6" width="29.6640625" customWidth="1"/>
+    <col min="7" max="7" width="18.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="7" customFormat="1">
@@ -5702,7 +5707,7 @@
       </c>
       <c r="H2" s="32"/>
     </row>
-    <row r="3" spans="1:8" ht="15.75">
+    <row r="3" spans="1:8" ht="15.6">
       <c r="A3" s="32">
         <v>1130589865</v>
       </c>
@@ -6034,16 +6039,16 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4DC1974-19B4-4A8B-940A-BAEC506B053A}">
   <dimension ref="B1:J169"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="51.28515625" customWidth="1"/>
-    <col min="2" max="2" width="28.140625" customWidth="1"/>
-    <col min="3" max="3" width="19.140625" customWidth="1"/>
-    <col min="4" max="4" width="19.42578125" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" customWidth="1"/>
-    <col min="6" max="6" width="41.42578125" customWidth="1"/>
-    <col min="7" max="7" width="34.42578125" customWidth="1"/>
-    <col min="8" max="8" width="14.28515625" customWidth="1"/>
+    <col min="1" max="1" width="51.33203125" customWidth="1"/>
+    <col min="2" max="2" width="28.109375" customWidth="1"/>
+    <col min="3" max="3" width="19.109375" customWidth="1"/>
+    <col min="4" max="4" width="19.44140625" customWidth="1"/>
+    <col min="5" max="5" width="15.33203125" customWidth="1"/>
+    <col min="6" max="6" width="41.44140625" customWidth="1"/>
+    <col min="7" max="7" width="34.44140625" customWidth="1"/>
+    <col min="8" max="8" width="14.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:10">

</xml_diff>